<commit_message>
Evaluate declared aggregate controls and bank trailer certification
contract.controls and source.control_file were schema-declared but never
executed — a silent PASS on the financial-totals layer. A new controls
stage recomputes counts, sums, min/max, null counts and distinct counts
(optionally grouped) over expected and target streams, compares them, and
certifies every declared control against the bank trailer file. The
workbook gains a Controls sheet and the demo seeds one; the source
generator emits the matching trailer.

Generated with [Devin](https://devin.ai)

Co-Authored-By: Devin <158243242+devin-ai-integration[bot]@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/data/mapping/bank_mapping.xlsx
+++ b/data/mapping/bank_mapping.xlsx
@@ -10,7 +10,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tables" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FieldMap" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mapping" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Controls" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mapping" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -420,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A24"/>
+  <dimension ref="A1:A30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="90" customWidth="1" min="1" max="1"/>
@@ -567,12 +568,50 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Connection details are NOT in this workbook — they live in</t>
+          <t>Controls sheet — aggregate controls (optional, financial totals).</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Type: count | sum | min | max | null_count | count_distinct.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Column / Group By name TARGET-side columns (comma-sep, max 3).</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  File Name: the certified total's name in the bank trailer file</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    (env source.control_file); blank = Control ID is used.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Connection details are NOT in this workbook — they live in</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
         <is>
           <t>config/environments/*.yaml; credentials come from env vars only.</t>
         </is>
@@ -2677,6 +2716,470 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:G14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Mapping ID</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Control ID</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Column</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Group By</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>File Name</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Enabled</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>customer_migration</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>customer_rows</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>customer_rows</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>customer_migration</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>null_phone</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>null_count</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>phone</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>null_phone</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>account_migration</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>account_rows</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>account_rows</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>account_migration</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>balance_total</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>sum</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>balance</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>balance_total</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>account_migration</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>balance_by_branch</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>sum</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>balance</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>branch_id</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>balance_by_branch</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>account_migration</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>distinct_customers</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>count_distinct</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>customer_id</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>distinct_customers</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>transaction_migration</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>txn_rows</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>txn_rows</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>transaction_migration</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>txn_amount_total</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>sum</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>amount</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr"/>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>txn_amount_total</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>transaction_migration</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>txn_by_type</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr"/>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>txn_type</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>txn_by_type</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>transaction_migration</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>max_txn</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>max</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>amount</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr"/>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>max_txn</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>loan_migration</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>loan_rows</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr"/>
+      <c r="E12" t="inlineStr"/>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>loan_rows</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>loan_migration</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>loan_balance_total</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>sum</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>current_balance</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr"/>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>loan_balance_total</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>branch_migration</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>branch_rows</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr"/>
+      <c r="E14" t="inlineStr"/>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>branch_rows</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:C20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>

</xml_diff>

<commit_message>
Check referential integrity across mappings on both sides
A Relations workbook sheet declares FK pairs (child column -> parent
column, target-side names). The relations stage builds canonical key sets
from each parent and counts exact orphan and null-FK totals in both the
source space (post-transform) and the target — so a child row that landed
without its parent, or a source-side orphan the migration would inherit,
fails instead of passing silently. Canonicalization keeps string
identifiers literal while unifying numeric int/float representations.

Generated with [Devin](https://devin.ai)

Co-Authored-By: Devin <158243242+devin-ai-integration[bot]@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/data/mapping/bank_mapping.xlsx
+++ b/data/mapping/bank_mapping.xlsx
@@ -11,7 +11,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tables" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FieldMap" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Controls" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mapping" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relations" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mapping" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -421,7 +422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A30"/>
+  <dimension ref="A1:A34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="90" customWidth="1" min="1" max="1"/>
@@ -606,12 +607,36 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Connection details are NOT in this workbook — they live in</t>
+          <t>Relations sheet — FK pairs across mappings (optional).</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Parent/Child columns are target-side names; every child value must</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  exist in the parent's column on BOTH source and target sides.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Connection details are NOT in this workbook — they live in</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
         <is>
           <t>config/environments/*.yaml; credentials come from env vars only.</t>
         </is>
@@ -3180,6 +3205,155 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:E5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Parent Mapping</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Parent Column</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Child Mapping</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Child Column</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Enabled</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>customer_migration</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>customer_id</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>account_migration</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>customer_id</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>branch_migration</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>branch_id</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>account_migration</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>branch_id</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>account_migration</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>account_id</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>transaction_migration</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>account_id</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>customer_migration</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>customer_id</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>loan_migration</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>customer_id</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:C20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>

</xml_diff>

<commit_message>
Evidence polish: transform-scoped compare, coverage gate, PII redaction
The transform stage now compares keys plus transform-derived columns only,
attributing drift to the transform layer instead of duplicating recon.
Validate Migration Evidence requires COMPLETE coverage, and
run.fail_on_unmapped turns unmapped source/target tables into failures.
The FieldMap PII column drives selective redaction — non-PII diff samples
show bounded values, PII and unknown columns stay redacted. The DQ stage
evaluates contract rules and key uniqueness in a single source pass.

Generated with [Devin](https://devin.ai)

Co-Authored-By: Devin <158243242+devin-ai-integration[bot]@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/data/mapping/bank_mapping.xlsx
+++ b/data/mapping/bank_mapping.xlsx
@@ -983,7 +983,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I44"/>
+  <dimension ref="A1:J44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1029,6 +1029,11 @@
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
+          <t>PII</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
           <t>Enabled</t>
         </is>
       </c>
@@ -1064,6 +1069,11 @@
       <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr">
         <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
           <t>yes</t>
         </is>
       </c>
@@ -1103,6 +1113,11 @@
       <c r="H3" t="inlineStr"/>
       <c r="I3" t="inlineStr">
         <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
           <t>yes</t>
         </is>
       </c>
@@ -1142,6 +1157,11 @@
       <c r="H4" t="inlineStr"/>
       <c r="I4" t="inlineStr">
         <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
           <t>yes</t>
         </is>
       </c>
@@ -1188,6 +1208,11 @@
           <t>yes</t>
         </is>
       </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1227,6 +1252,11 @@
         </is>
       </c>
       <c r="I6" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
@@ -1267,6 +1297,11 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
           <t>yes</t>
         </is>
       </c>
@@ -1309,6 +1344,11 @@
         </is>
       </c>
       <c r="I8" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
@@ -1352,6 +1392,11 @@
           <t>yes</t>
         </is>
       </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1391,6 +1436,11 @@
         </is>
       </c>
       <c r="I10" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
@@ -1431,6 +1481,11 @@
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr">
         <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
           <t>yes</t>
         </is>
       </c>
@@ -1470,6 +1525,11 @@
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr">
         <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
           <t>yes</t>
         </is>
       </c>
@@ -1512,6 +1572,11 @@
           <t>yes</t>
         </is>
       </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1551,6 +1616,11 @@
         </is>
       </c>
       <c r="I14" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
@@ -1587,6 +1657,11 @@
       <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr">
         <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
           <t>yes</t>
         </is>
       </c>
@@ -1622,6 +1697,11 @@
       <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr">
         <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
           <t>yes</t>
         </is>
       </c>
@@ -1657,6 +1737,11 @@
       <c r="H17" t="inlineStr"/>
       <c r="I17" t="inlineStr">
         <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
           <t>yes</t>
         </is>
       </c>
@@ -1696,6 +1781,11 @@
       <c r="H18" t="inlineStr"/>
       <c r="I18" t="inlineStr">
         <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
           <t>yes</t>
         </is>
       </c>
@@ -1738,6 +1828,11 @@
         </is>
       </c>
       <c r="I19" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
@@ -1774,6 +1869,11 @@
       <c r="H20" t="inlineStr"/>
       <c r="I20" t="inlineStr">
         <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
           <t>yes</t>
         </is>
       </c>
@@ -1809,6 +1909,11 @@
       <c r="H21" t="inlineStr"/>
       <c r="I21" t="inlineStr">
         <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
           <t>yes</t>
         </is>
       </c>
@@ -1852,6 +1957,11 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
           <t>yes</t>
         </is>
       </c>
@@ -1894,6 +2004,11 @@
         </is>
       </c>
       <c r="I23" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
@@ -1930,6 +2045,11 @@
       <c r="H24" t="inlineStr"/>
       <c r="I24" t="inlineStr">
         <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
           <t>yes</t>
         </is>
       </c>
@@ -1965,6 +2085,11 @@
       <c r="H25" t="inlineStr"/>
       <c r="I25" t="inlineStr">
         <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
           <t>yes</t>
         </is>
       </c>
@@ -2000,6 +2125,11 @@
       <c r="H26" t="inlineStr"/>
       <c r="I26" t="inlineStr">
         <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
           <t>yes</t>
         </is>
       </c>
@@ -2039,6 +2169,11 @@
       <c r="H27" t="inlineStr"/>
       <c r="I27" t="inlineStr">
         <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
           <t>yes</t>
         </is>
       </c>
@@ -2082,6 +2217,11 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
           <t>yes</t>
         </is>
       </c>
@@ -2125,6 +2265,11 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
           <t>yes</t>
         </is>
       </c>
@@ -2167,6 +2312,11 @@
         </is>
       </c>
       <c r="I30" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
@@ -2203,6 +2353,11 @@
       <c r="H31" t="inlineStr"/>
       <c r="I31" t="inlineStr">
         <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
           <t>yes</t>
         </is>
       </c>
@@ -2238,6 +2393,11 @@
       <c r="H32" t="inlineStr"/>
       <c r="I32" t="inlineStr">
         <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
           <t>yes</t>
         </is>
       </c>
@@ -2281,6 +2441,11 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
           <t>yes</t>
         </is>
       </c>
@@ -2324,6 +2489,11 @@
       </c>
       <c r="I34" t="inlineStr">
         <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
           <t>yes</t>
         </is>
       </c>
@@ -2367,6 +2537,11 @@
       </c>
       <c r="I35" t="inlineStr">
         <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
           <t>yes</t>
         </is>
       </c>
@@ -2409,6 +2584,11 @@
         </is>
       </c>
       <c r="I36" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
@@ -2445,6 +2625,11 @@
       <c r="H37" t="inlineStr"/>
       <c r="I37" t="inlineStr">
         <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
           <t>yes</t>
         </is>
       </c>
@@ -2480,6 +2665,11 @@
       <c r="H38" t="inlineStr"/>
       <c r="I38" t="inlineStr">
         <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
           <t>yes</t>
         </is>
       </c>
@@ -2522,6 +2712,11 @@
         </is>
       </c>
       <c r="I39" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
@@ -2558,6 +2753,11 @@
       <c r="H40" t="inlineStr"/>
       <c r="I40" t="inlineStr">
         <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
           <t>yes</t>
         </is>
       </c>
@@ -2601,6 +2801,11 @@
       </c>
       <c r="I41" t="inlineStr">
         <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
           <t>yes</t>
         </is>
       </c>
@@ -2643,6 +2848,11 @@
         </is>
       </c>
       <c r="I42" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
@@ -2683,6 +2893,11 @@
       <c r="H43" t="inlineStr"/>
       <c r="I43" t="inlineStr">
         <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
           <t>yes</t>
         </is>
       </c>
@@ -2725,6 +2940,11 @@
         </is>
       </c>
       <c r="I44" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
         <is>
           <t>yes</t>
         </is>

</xml_diff>